<commit_message>
phase 2: overlap + coverage passes, thin-canon report, 23 proposed rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSXofh6XbF2HBYEMwgkCSz
</commit_message>
<xml_diff>
--- a/google-ads-skills-index.xlsx
+++ b/google-ads-skills-index.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S91"/>
+  <dimension ref="A1:S114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
@@ -8468,42 +8468,1675 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="15" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="16" t="inlineStr">
+        <is>
+          <t>Full account audit — multi-module diagnostic</t>
+        </is>
+      </c>
+      <c r="C92" s="15" t="inlineStr">
+        <is>
+          <t>Testing &amp; measurement</t>
+        </is>
+      </c>
+      <c r="D92" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E92" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F92" s="15" t="inlineStr">
+        <is>
+          <t>Diagnose</t>
+        </is>
+      </c>
+      <c r="G92" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H92" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I92" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J92" s="16" t="inlineStr">
+        <is>
+          <t>Taking over an account, quarterly review, or pre-pitch; need a ranked list of critical issues across tracking, structure, settings, keywords/search terms, bids/budgets, ads, landing pages</t>
+        </is>
+      </c>
+      <c r="K92" s="15" t="inlineStr">
+        <is>
+          <t>Practitioner method</t>
+        </is>
+      </c>
+      <c r="L92" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M92" s="15" t="n"/>
+      <c r="N92" s="17" t="n"/>
+      <c r="O92" s="15" t="inlineStr">
+        <is>
+          <t>why core: PPC OS public hub exposes 'Account Audit — 24 diagnostics across 5 modules' and an Account Health Report (Tracking, Campaign Structure, Landing Pages, QS, Ad Quality); TPE #149 lists 13 stacked audits; Hopkins (SEJ 2025) on regular audits; Optmyzr 9-section audit. Library has per-topic diagnostics but no library-level audit row.</t>
+        </is>
+      </c>
+      <c r="P92" s="15" t="n"/>
+      <c r="Q92" s="16" t="n"/>
+      <c r="R92" s="15" t="n"/>
+      <c r="S92" s="15" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="15" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>Conversion tracking audit</t>
+        </is>
+      </c>
+      <c r="C93" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E93" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F93" s="15" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="G93" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H93" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I93" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J93" s="16" t="inlineStr">
+        <is>
+          <t>Before trusting Smart Bidding on any account: verify tags, primary/secondary actions, duplicates, attribution, Enhanced Conversions, Consent Mode v2, OCI, counting method</t>
+        </is>
+      </c>
+      <c r="K93" s="15" t="inlineStr">
+        <is>
+          <t>Practitioner method</t>
+        </is>
+      </c>
+      <c r="L93" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M93" s="15" t="n"/>
+      <c r="N93" s="17" t="n"/>
+      <c r="O93" s="15" t="inlineStr">
+        <is>
+          <t>why core: PPC OS public hub 'Tracking Audit — 50-point check' naming Enhanced Conversions, Consent Mode v2, OCI, attribution model, duplicate actions, primary/secondary; ZATO 'Conversion tracking: why clean data is everything'; Hopkins SEJ 2024 enterprise tracking pitfalls. Rows 47/48 cover two pieces only.</t>
+        </is>
+      </c>
+      <c r="P93" s="15" t="n"/>
+      <c r="Q93" s="16" t="n"/>
+      <c r="R93" s="15" t="n"/>
+      <c r="S93" s="15" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="15" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="16" t="inlineStr">
+        <is>
+          <t>Weekly account review routine</t>
+        </is>
+      </c>
+      <c r="C94" s="15" t="inlineStr">
+        <is>
+          <t>Testing &amp; measurement</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E94" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F94" s="15" t="inlineStr">
+        <is>
+          <t>Optimise</t>
+        </is>
+      </c>
+      <c r="G94" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H94" s="15" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="I94" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J94" s="16" t="inlineStr">
+        <is>
+          <t>Running the standing weekly check: what to look at, in what order, over which lookbacks, and what triggers an action vs a watch</t>
+        </is>
+      </c>
+      <c r="K94" s="15" t="inlineStr">
+        <is>
+          <t>Practitioner method</t>
+        </is>
+      </c>
+      <c r="L94" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M94" s="15" t="n"/>
+      <c r="N94" s="17" t="n"/>
+      <c r="O94" s="15" t="inlineStr">
+        <is>
+          <t>why core: PPC OS 'Performance Analysis' with sample output 'Weekly Review' and 7/30/90/365-day trend windows (TPE #149); Optmyzr audit cadence (weekly health / monthly / quarterly); Adalysis 'how to automate your Google Ads KPI monitoring'.</t>
+        </is>
+      </c>
+      <c r="P94" s="15" t="n"/>
+      <c r="Q94" s="16" t="n"/>
+      <c r="R94" s="15" t="n"/>
+      <c r="S94" s="15" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="15" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="16" t="inlineStr">
+        <is>
+          <t>Performance change root-cause diagnosis</t>
+        </is>
+      </c>
+      <c r="C95" s="15" t="inlineStr">
+        <is>
+          <t>Testing &amp; measurement</t>
+        </is>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E95" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F95" s="15" t="inlineStr">
+        <is>
+          <t>Diagnose</t>
+        </is>
+      </c>
+      <c r="G95" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H95" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I95" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J95" s="16" t="inlineStr">
+        <is>
+          <t>CPC, CTR, clicks, conversions or CPA moved and nobody knows why; need a decomposition tree before touching anything</t>
+        </is>
+      </c>
+      <c r="K95" s="15" t="inlineStr">
+        <is>
+          <t>Adalysis KPI monitoring series</t>
+        </is>
+      </c>
+      <c r="L95" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M95" s="15" t="n"/>
+      <c r="N95" s="17" t="n"/>
+      <c r="O95" s="15" t="inlineStr">
+        <is>
+          <t>why core: Adalysis 'KPI monitoring diagnosis' series (why does CPC/cost, CTR, clicks, conversions/CVR, impression volume change) plus 'analyze the correct time periods'; PPC OS 'Performance Analysis — the why behind metric shifts'. Rows 84/83/49 cover single causes only.</t>
+        </is>
+      </c>
+      <c r="P95" s="15" t="n"/>
+      <c r="Q95" s="16" t="n"/>
+      <c r="R95" s="15" t="n"/>
+      <c r="S95" s="15" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="15" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>Bid strategy selection — Smart Bidding vs manual, target vs maximise</t>
+        </is>
+      </c>
+      <c r="C96" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="E96" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F96" s="15" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="G96" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H96" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I96" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J96" s="16" t="inlineStr">
+        <is>
+          <t>Choosing or changing a bid strategy per campaign; deciding whether volume, signal quality and spend-control needs justify Smart Bidding at all</t>
+        </is>
+      </c>
+      <c r="K96" s="15" t="inlineStr">
+        <is>
+          <t>Optmyzr / Adalysis / PPC Mastery</t>
+        </is>
+      </c>
+      <c r="L96" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M96" s="15" t="n"/>
+      <c r="N96" s="17" t="n"/>
+      <c r="O96" s="15" t="inlineStr">
+        <is>
+          <t>why core: Vallaeys 'When to stop using Smart Bidding' (Optmyzr, May 2026; ~50 conv/30d rule, manual CPC + rules alternative); Adalysis 'when to use target vs max CPA/ROAS'; PPC Mastery lists bid strategy choice as a core topic; Hopkins SEJ budget-by-stage. No existing row covers the choice itself.</t>
+        </is>
+      </c>
+      <c r="P96" s="15" t="n"/>
+      <c r="Q96" s="16" t="n"/>
+      <c r="R96" s="15" t="n"/>
+      <c r="S96" s="15" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="16" t="inlineStr">
+        <is>
+          <t>Targets from unit economics — break-even ROAS, profit curve, growth vs efficiency</t>
+        </is>
+      </c>
+      <c r="C97" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D97" s="15" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="E97" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F97" s="15" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="G97" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H97" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I97" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J97" s="16" t="inlineStr">
+        <is>
+          <t>Setting or renegotiating tCPA/tROAS with a client; need margin, LTV, payback and a primary-goal/guardrail pair before touching the target</t>
+        </is>
+      </c>
+      <c r="K97" s="15" t="inlineStr">
+        <is>
+          <t>Mike Rhodes / PPC Mastery</t>
+        </is>
+      </c>
+      <c r="L97" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M97" s="15" t="n"/>
+      <c r="N97" s="17" t="n"/>
+      <c r="O97" s="15" t="inlineStr">
+        <is>
+          <t>why core: Rhodes 8020agent (profit curve, budget optimisation, break-even ROAS); PPC OS course 'Goal Setting Mastery' + vault 'target calculators'; TPE #144 growth vs efficiency (primary focus + guardrail), TPE #148 LTV flywheel, TPE #149 Phase 1 context questions; Optmyzr ROAS-by-vertical benchmarks (Sep 2026).</t>
+        </is>
+      </c>
+      <c r="P97" s="15" t="n"/>
+      <c r="Q97" s="16" t="n"/>
+      <c r="R97" s="15" t="n"/>
+      <c r="S97" s="15" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="15" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="16" t="inlineStr">
+        <is>
+          <t>Smart Bidding learning period — what resets it and change-size rules</t>
+        </is>
+      </c>
+      <c r="C98" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F98" s="15" t="inlineStr">
+        <is>
+          <t>Optimise</t>
+        </is>
+      </c>
+      <c r="G98" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H98" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I98" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J98" s="16" t="inlineStr">
+        <is>
+          <t>Planning any target, budget, structure or conversion-action change on a Smart Bidding campaign; deciding step size and spacing to avoid relearning</t>
+        </is>
+      </c>
+      <c r="K98" s="15" t="inlineStr">
+        <is>
+          <t>Practitioner method</t>
+        </is>
+      </c>
+      <c r="L98" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M98" s="15" t="n"/>
+      <c r="N98" s="17" t="n"/>
+      <c r="O98" s="15" t="inlineStr">
+        <is>
+          <t>why core: Hopkins 'What are learning periods' (SEJ, Dec 2025) and 'Why do budgets overspend with tROAS' (Feb 2026); Adalysis 'what happens when you change your PPC budgets'; PPC Mastery structure-under-Smart-Bidding material. Row 9 only covers campaigns stuck in learning from low volume.</t>
+        </is>
+      </c>
+      <c r="P98" s="15" t="n"/>
+      <c r="Q98" s="16" t="n"/>
+      <c r="R98" s="15" t="n"/>
+      <c r="S98" s="15" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="15" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="16" t="inlineStr">
+        <is>
+          <t>AI Max for Search — test design and evaluation</t>
+        </is>
+      </c>
+      <c r="C99" s="15" t="inlineStr">
+        <is>
+          <t>Keyword &amp; query</t>
+        </is>
+      </c>
+      <c r="D99" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E99" s="15" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="F99" s="15" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="G99" s="15" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="H99" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I99" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J99" s="16" t="inlineStr">
+        <is>
+          <t>Google is pushing AI Max; need prerequisites, a limited test, and how to read search terms, asset source and URL expansion before keeping it on</t>
+        </is>
+      </c>
+      <c r="K99" s="15" t="inlineStr">
+        <is>
+          <t>Adalysis / ZATO</t>
+        </is>
+      </c>
+      <c r="L99" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M99" s="15" t="n"/>
+      <c r="N99" s="17" t="n"/>
+      <c r="O99" s="15" t="inlineStr">
+        <is>
+          <t>why core: Geddes 'How to evaluate your AI Max performance' (Adalysis, Aug 2026; broad-match prerequisite, 30 conv/mo, n-gram + asset-source + URL analysis); ZATO has a whole 'AI Max for Search' topic; Cruz 'What are you optimizing for when keywords matter less' (SEL, Apr 2026). No row mentions AI Max.</t>
+        </is>
+      </c>
+      <c r="P99" s="15" t="n"/>
+      <c r="Q99" s="16" t="n"/>
+      <c r="R99" s="15" t="n"/>
+      <c r="S99" s="15" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="15" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="16" t="inlineStr">
+        <is>
+          <t>Product performance bucketing for Shopping and PMax</t>
+        </is>
+      </c>
+      <c r="C100" s="15" t="inlineStr">
+        <is>
+          <t>Shopping &amp; feeds</t>
+        </is>
+      </c>
+      <c r="D100" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E100" s="15" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="F100" s="15" t="inlineStr">
+        <is>
+          <t>Optimise</t>
+        </is>
+      </c>
+      <c r="G100" s="15" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="H100" s="15" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I100" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J100" s="16" t="inlineStr">
+        <is>
+          <t>Spend concentrated on a few SKUs while most products get no impressions; want zombies/heroes/sidekicks split into campaigns or asset groups</t>
+        </is>
+      </c>
+      <c r="K100" s="15" t="inlineStr">
+        <is>
+          <t>Mike Rhodes / Optmyzr</t>
+        </is>
+      </c>
+      <c r="L100" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M100" s="15" t="n"/>
+      <c r="N100" s="17" t="n"/>
+      <c r="O100" s="15" t="inlineStr">
+        <is>
+          <t>why core: Rhodes 'products' and 'check-product-data' scripts (GitHub mikerhodesideas/free); Optmyzr 'segment products in Google Shopping ads'; PPC OS 'shopping feed and product optimization'. Row 64 tiers by margin/stock, not by performance.</t>
+        </is>
+      </c>
+      <c r="P100" s="15" t="n"/>
+      <c r="Q100" s="16" t="n"/>
+      <c r="R100" s="15" t="n"/>
+      <c r="S100" s="15" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="16" t="inlineStr">
+        <is>
+          <t>Bid adjustments under Smart Bidding — what still applies</t>
+        </is>
+      </c>
+      <c r="C101" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D101" s="15" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="E101" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F101" s="15" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="G101" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H101" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I101" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J101" s="16" t="inlineStr">
+        <is>
+          <t>Inherited account full of device/location/schedule/audience adjustments on tCPA/tROAS; deciding what to strip, what -100% exclusions remain valid</t>
+        </is>
+      </c>
+      <c r="K101" s="15" t="inlineStr">
+        <is>
+          <t>PPC Mastery / Adalysis</t>
+        </is>
+      </c>
+      <c r="L101" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M101" s="15" t="n"/>
+      <c r="N101" s="17" t="n"/>
+      <c r="O101" s="15" t="inlineStr">
+        <is>
+          <t>why core: TPE #145 'Why bid adjustments are dead' (public cheat-sheet by strategy); Adalysis 'how bid adjustments are used by bidding method' and 'how audience bid adjustments work with tCPA/tROAS'. Row 41 covers value rules only.</t>
+        </is>
+      </c>
+      <c r="P101" s="15" t="n"/>
+      <c r="Q101" s="16" t="n"/>
+      <c r="R101" s="15" t="n"/>
+      <c r="S101" s="15" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="15" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="16" t="inlineStr">
+        <is>
+          <t>Budget reallocation across campaigns by marginal return</t>
+        </is>
+      </c>
+      <c r="C102" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D102" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E102" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F102" s="15" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="G102" s="15" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="H102" s="15" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I102" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J102" s="16" t="inlineStr">
+        <is>
+          <t>Fixed account budget; some campaigns limited by budget, others underspending; deciding where the next euro goes and whether shared budgets help</t>
+        </is>
+      </c>
+      <c r="K102" s="15" t="inlineStr">
+        <is>
+          <t>Practitioner method</t>
+        </is>
+      </c>
+      <c r="L102" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M102" s="15" t="n"/>
+      <c r="N102" s="17" t="n"/>
+      <c r="O102" s="15" t="inlineStr">
+        <is>
+          <t>why core: PPC OS 'Bids &amp; Budgets — reallocates budgets, validates targets'; Optmyzr 'manage PPC budgets' and 'smart bidding budget caps guide'; Adalysis 'why your campaigns are underspending' and 'IS loss due to budget'; Rhodes 8020agent budget optimiser. Row 71 is only the pacing alert.</t>
+        </is>
+      </c>
+      <c r="P102" s="15" t="n"/>
+      <c r="Q102" s="16" t="n"/>
+      <c r="R102" s="15" t="n"/>
+      <c r="S102" s="15" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="15" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="16" t="inlineStr">
+        <is>
+          <t>Scaling without breaking efficiency — budget and target step rules</t>
+        </is>
+      </c>
+      <c r="C103" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D103" s="15" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="E103" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F103" s="15" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="G103" s="15" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="H103" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I103" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J103" s="16" t="inlineStr">
+        <is>
+          <t>Client wants 2x volume; deciding the order of levers (budget, target, match type, campaign type) and step sizes without CPA blowing up</t>
+        </is>
+      </c>
+      <c r="K103" s="15" t="inlineStr">
+        <is>
+          <t>ZATO / PPC Mastery</t>
+        </is>
+      </c>
+      <c r="L103" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M103" s="15" t="n"/>
+      <c r="N103" s="17" t="n"/>
+      <c r="O103" s="15" t="inlineStr">
+        <is>
+          <t>why core: ZATO 'How to scale Google Ads' and 'The physics of PPC'; TPE #147 bottom-up funnel, #144 growth vs efficiency; Hopkins 'From launch to scale: budget strategies for all campaign stages' (SEJ 2024).</t>
+        </is>
+      </c>
+      <c r="P103" s="15" t="n"/>
+      <c r="Q103" s="16" t="n"/>
+      <c r="R103" s="15" t="n"/>
+      <c r="S103" s="15" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="15" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="16" t="inlineStr">
+        <is>
+          <t>Campaign not serving / zero impressions troubleshooting</t>
+        </is>
+      </c>
+      <c r="C104" s="15" t="inlineStr">
+        <is>
+          <t>Testing &amp; measurement</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E104" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F104" s="15" t="inlineStr">
+        <is>
+          <t>Diagnose</t>
+        </is>
+      </c>
+      <c r="G104" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H104" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I104" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J104" s="16" t="inlineStr">
+        <is>
+          <t>Live campaign with no or near-zero impressions; need the ordered checklist (billing, policy, status, targeting, bids/targets, negatives, eligibility) before escalating</t>
+        </is>
+      </c>
+      <c r="K104" s="15" t="inlineStr">
+        <is>
+          <t>ZATO / Navah Hopkins</t>
+        </is>
+      </c>
+      <c r="L104" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M104" s="15" t="n"/>
+      <c r="N104" s="17" t="n"/>
+      <c r="O104" s="15" t="inlineStr">
+        <is>
+          <t>why core: ZATO 'Why isn't my campaign serving — the most asked question in the support forum'; Hopkins 'Why have my ads not got any impressions' (SEJ 2024). Rows 46 and 19 cover under-delivery and low-volume keywords, not non-serving.</t>
+        </is>
+      </c>
+      <c r="P104" s="15" t="n"/>
+      <c r="Q104" s="16" t="n"/>
+      <c r="R104" s="15" t="n"/>
+      <c r="S104" s="15" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="15" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="16" t="inlineStr">
+        <is>
+          <t>New Search campaign launch checklist and first-30-days watch</t>
+        </is>
+      </c>
+      <c r="C105" s="15" t="inlineStr">
+        <is>
+          <t>Account structure</t>
+        </is>
+      </c>
+      <c r="D105" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E105" s="15" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="F105" s="15" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="G105" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H105" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I105" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J105" s="16" t="inlineStr">
+        <is>
+          <t>Launching a new Search campaign; pre-launch settings check and what to review in weeks 1–2 (relevance, net-new impressions, IS) vs weeks 3–4 (conversion quality, serving, match type, bid method switch)</t>
+        </is>
+      </c>
+      <c r="K105" s="15" t="inlineStr">
+        <is>
+          <t>Adalysis / PPC Mastery</t>
+        </is>
+      </c>
+      <c r="L105" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M105" s="15" t="n"/>
+      <c r="N105" s="17" t="n"/>
+      <c r="O105" s="15" t="inlineStr">
+        <is>
+          <t>why core: Geddes 'Launching a new Search campaign: what to watch in the first month' (Adalysis, 2025); PPC OS 'Search Mastery' public course lists a launch checklist. Rows 87/88 are settings only.</t>
+        </is>
+      </c>
+      <c r="P105" s="15" t="n"/>
+      <c r="Q105" s="16" t="n"/>
+      <c r="R105" s="15" t="n"/>
+      <c r="S105" s="15" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="15" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="16" t="inlineStr">
+        <is>
+          <t>Ad assets (sitelinks, callouts, snippets, images) — build and evaluate</t>
+        </is>
+      </c>
+      <c r="C106" s="15" t="inlineStr">
+        <is>
+          <t>RSA &amp; ad copy</t>
+        </is>
+      </c>
+      <c r="D106" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E106" s="15" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="F106" s="15" t="inlineStr">
+        <is>
+          <t>Optimise</t>
+        </is>
+      </c>
+      <c r="G106" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H106" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I106" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J106" s="16" t="inlineStr">
+        <is>
+          <t>Setting up or auditing assets; reading asset-level performance and the asset-vs-ad report; which assets to pin to campaign vs account level</t>
+        </is>
+      </c>
+      <c r="K106" s="15" t="inlineStr">
+        <is>
+          <t>Adalysis</t>
+        </is>
+      </c>
+      <c r="L106" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M106" s="15" t="n"/>
+      <c r="N106" s="17" t="n"/>
+      <c r="O106" s="15" t="inlineStr">
+        <is>
+          <t>why core: Adalysis 'understanding and analyzing extension data', 'easily analyze ad extension usage', 'importance of ad extensions', '20 more sitelink ideas'; PPC OS 'Ad Quality (RSAs)' health sub-score. The library has no row on assets/extensions.</t>
+        </is>
+      </c>
+      <c r="P106" s="15" t="n"/>
+      <c r="Q106" s="16" t="n"/>
+      <c r="R106" s="15" t="n"/>
+      <c r="S106" s="15" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="15" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="16" t="inlineStr">
+        <is>
+          <t>Feed attribute optimisation beyond titles (product_type, google_product_category, id, description)</t>
+        </is>
+      </c>
+      <c r="C107" s="15" t="inlineStr">
+        <is>
+          <t>Shopping &amp; feeds</t>
+        </is>
+      </c>
+      <c r="D107" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E107" s="15" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="F107" s="15" t="inlineStr">
+        <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="G107" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H107" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I107" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J107" s="16" t="inlineStr">
+        <is>
+          <t>Titles done; want the secondary attributes that drive matching and segmentation right, and stable product IDs before any feed-provider change</t>
+        </is>
+      </c>
+      <c r="K107" s="15" t="inlineStr">
+        <is>
+          <t>ZATO Merchant Center Mastery</t>
+        </is>
+      </c>
+      <c r="L107" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M107" s="15" t="n"/>
+      <c r="N107" s="17" t="n"/>
+      <c r="O107" s="15" t="inlineStr">
+        <is>
+          <t>why core: ZATO 'optimize product_type', 'optimize google_product_category', 'why the id attribute matters', 'optimize product descriptions (2026)', 'changing feed providers: roadmap'; PPC OS 'Feeds — titles and secondary attributes'. Rows 65/66 cover rules mechanics and titles only.</t>
+        </is>
+      </c>
+      <c r="P107" s="15" t="n"/>
+      <c r="Q107" s="16" t="n"/>
+      <c r="R107" s="15" t="n"/>
+      <c r="S107" s="15" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="15" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="16" t="inlineStr">
+        <is>
+          <t>Merchant Center account suspension recovery</t>
+        </is>
+      </c>
+      <c r="C108" s="15" t="inlineStr">
+        <is>
+          <t>Shopping &amp; feeds</t>
+        </is>
+      </c>
+      <c r="D108" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E108" s="15" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="F108" s="15" t="inlineStr">
+        <is>
+          <t>Protect</t>
+        </is>
+      </c>
+      <c r="G108" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H108" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I108" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J108" s="16" t="inlineStr">
+        <is>
+          <t>Account-level suspension (misrepresentation, unacceptable business practices, tax/shipping) rather than item disapprovals; need the compliance checklist and appeal sequence</t>
+        </is>
+      </c>
+      <c r="K108" s="15" t="inlineStr">
+        <is>
+          <t>ZATO</t>
+        </is>
+      </c>
+      <c r="L108" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M108" s="15" t="n"/>
+      <c r="N108" s="17" t="n"/>
+      <c r="O108" s="15" t="inlineStr">
+        <is>
+          <t>why core: ZATO 'How to fix a Merchant Center suspension for misrepresentation', 'tax suspension fix', 'preventing disapprovals and suspensions by mastering compliance'. Row 67 is item-level disapprovals.</t>
+        </is>
+      </c>
+      <c r="P108" s="15" t="n"/>
+      <c r="Q108" s="16" t="n"/>
+      <c r="R108" s="15" t="n"/>
+      <c r="S108" s="15" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="16" t="inlineStr">
+        <is>
+          <t>PMax asset group and asset performance review</t>
+        </is>
+      </c>
+      <c r="C109" s="15" t="inlineStr">
+        <is>
+          <t>Performance Max</t>
+        </is>
+      </c>
+      <c r="D109" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E109" s="15" t="inlineStr">
+        <is>
+          <t>PMax</t>
+        </is>
+      </c>
+      <c r="F109" s="15" t="inlineStr">
+        <is>
+          <t>Optimise</t>
+        </is>
+      </c>
+      <c r="G109" s="15" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="H109" s="15" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I109" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J109" s="16" t="inlineStr">
+        <is>
+          <t>Deciding which assets and asset groups to replace; reading asset ratings, asset-group spend and conversion split, and auto-generated vs supplied assets</t>
+        </is>
+      </c>
+      <c r="K109" s="15" t="inlineStr">
+        <is>
+          <t>Mike Rhodes</t>
+        </is>
+      </c>
+      <c r="L109" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M109" s="15" t="n"/>
+      <c r="N109" s="17" t="n"/>
+      <c r="O109" s="15" t="inlineStr">
+        <is>
+          <t>why core: Rhodes 'pmax-assets' script (GitHub); PPC OS 'pMax' skill and 'Performance Max Mastery' course; Hopkins 'Should you use auto-generated creative' (SEJ 2026). Row 58 is structure only.</t>
+        </is>
+      </c>
+      <c r="P109" s="15" t="n"/>
+      <c r="Q109" s="16" t="n"/>
+      <c r="R109" s="15" t="n"/>
+      <c r="S109" s="15" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="15" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="16" t="inlineStr">
+        <is>
+          <t>Spam conversions and invalid traffic polluting Smart Bidding</t>
+        </is>
+      </c>
+      <c r="C110" s="15" t="inlineStr">
+        <is>
+          <t>Bidding</t>
+        </is>
+      </c>
+      <c r="D110" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E110" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F110" s="15" t="inlineStr">
+        <is>
+          <t>Protect</t>
+        </is>
+      </c>
+      <c r="G110" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H110" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I110" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J110" s="16" t="inlineStr">
+        <is>
+          <t>Sudden conversion spike with no revenue, bot form fills, or suspected click fraud; detect, confirm, negate/exclude, and clean the bidding signal</t>
+        </is>
+      </c>
+      <c r="K110" s="15" t="inlineStr">
+        <is>
+          <t>Practitioner method</t>
+        </is>
+      </c>
+      <c r="L110" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M110" s="15" t="n"/>
+      <c r="N110" s="17" t="n"/>
+      <c r="O110" s="15" t="inlineStr">
+        <is>
+          <t>why core: Hopkins 'How to identify and solve click fraud' (SEJ, Apr 2026); Optmyzr 'Protect Smart Bidding from spam conversions' (Jul 2026, method only, vendor byline); ZATO clean-data post. Row 44 covers data exclusions after the fact, not detection.</t>
+        </is>
+      </c>
+      <c r="P110" s="15" t="n"/>
+      <c r="Q110" s="16" t="n"/>
+      <c r="R110" s="15" t="n"/>
+      <c r="S110" s="15" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="15" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="16" t="inlineStr">
+        <is>
+          <t>Landing page audit for paid search</t>
+        </is>
+      </c>
+      <c r="C111" s="15" t="inlineStr">
+        <is>
+          <t>Quality Score</t>
+        </is>
+      </c>
+      <c r="D111" s="15" t="inlineStr">
+        <is>
+          <t>Technique</t>
+        </is>
+      </c>
+      <c r="E111" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F111" s="15" t="inlineStr">
+        <is>
+          <t>Optimise</t>
+        </is>
+      </c>
+      <c r="G111" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H111" s="15" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="I111" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J111" s="16" t="inlineStr">
+        <is>
+          <t>CVR low despite relevant traffic; structured LP audit (message match, hero, proof, speed, form/CTA, guarantee) and how to test LP with ad together</t>
+        </is>
+      </c>
+      <c r="K111" s="15" t="inlineStr">
+        <is>
+          <t>PPC Mastery / Adalysis</t>
+        </is>
+      </c>
+      <c r="L111" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M111" s="15" t="n"/>
+      <c r="N111" s="17" t="n"/>
+      <c r="O111" s="15" t="inlineStr">
+        <is>
+          <t>why core: PPC OS 'Landing Pages — 6-pillar structural audit' and 'Landing Page Mastery' course; Adalysis 'test landing pages and ads together', 'customer journey testing'; Rhodes 'landing-page' script; Optmyzr 'PPC landing page AI signal problem'. Row 36 is the QS LPE component only.</t>
+        </is>
+      </c>
+      <c r="P111" s="15" t="n"/>
+      <c r="Q111" s="16" t="n"/>
+      <c r="R111" s="15" t="n"/>
+      <c r="S111" s="15" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="15" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="16" t="inlineStr">
+        <is>
+          <t>Automation layering — guardrail automations over Google's automation</t>
+        </is>
+      </c>
+      <c r="C112" s="15" t="inlineStr">
+        <is>
+          <t>Scripts &amp; automation</t>
+        </is>
+      </c>
+      <c r="D112" s="15" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="E112" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F112" s="15" t="inlineStr">
+        <is>
+          <t>Optimise</t>
+        </is>
+      </c>
+      <c r="G112" s="15" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="H112" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I112" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J112" s="16" t="inlineStr">
+        <is>
+          <t>Deciding which Google automations to adopt and which monitors (alerts, rules, scripts) must sit on top of each before go-live</t>
+        </is>
+      </c>
+      <c r="K112" s="15" t="inlineStr">
+        <is>
+          <t>Fred Vallaeys</t>
+        </is>
+      </c>
+      <c r="L112" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M112" s="15" t="n"/>
+      <c r="N112" s="17" t="n"/>
+      <c r="O112" s="15" t="inlineStr">
+        <is>
+          <t>why core: Vallaeys 'Automation layering is driving PPC' (SEL) and canon lists it among his strongest topics; Hopkins 'How do I keep control as platforms automate my account' (SEJ, Sep 2026); Optmyzr 72,358-account manual-work study (Sep 2026). Row 77 is rules-vs-scripts tool choice, not the layering strategy.</t>
+        </is>
+      </c>
+      <c r="P112" s="15" t="n"/>
+      <c r="Q112" s="16" t="n"/>
+      <c r="R112" s="15" t="n"/>
+      <c r="S112" s="15" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="15" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="16" t="inlineStr">
+        <is>
+          <t>Change history monitoring</t>
+        </is>
+      </c>
+      <c r="C113" s="15" t="inlineStr">
+        <is>
+          <t>Scripts &amp; automation</t>
+        </is>
+      </c>
+      <c r="D113" s="15" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="E113" s="15" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F113" s="15" t="inlineStr">
+        <is>
+          <t>Protect</t>
+        </is>
+      </c>
+      <c r="G113" s="15" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H113" s="15" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="I113" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J113" s="16" t="inlineStr">
+        <is>
+          <t>Multiple users, Google reps or auto-apply touching the account; want daily alerts on unexpected changes with who/what</t>
+        </is>
+      </c>
+      <c r="K113" s="15" t="inlineStr">
+        <is>
+          <t>Nils Rooijmans</t>
+        </is>
+      </c>
+      <c r="L113" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M113" s="15" t="n"/>
+      <c r="N113" s="17" t="n"/>
+      <c r="O113" s="15" t="inlineStr">
+        <is>
+          <t>why core: Nils 'Change history alerts' script (public catalogue); Hopkins Sep 2026 on keeping control under automation. Row 78 only opts out of auto-apply; it does not monitor what changed.</t>
+        </is>
+      </c>
+      <c r="P113" s="15" t="n"/>
+      <c r="Q113" s="16" t="n"/>
+      <c r="R113" s="15" t="n"/>
+      <c r="S113" s="15" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="15" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="16" t="inlineStr">
+        <is>
+          <t>Lin-Rodnitzky ratio as a search-term health metric</t>
+        </is>
+      </c>
+      <c r="C114" s="15" t="inlineStr">
+        <is>
+          <t>Keyword &amp; query</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="E114" s="15" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="F114" s="15" t="inlineStr">
+        <is>
+          <t>Diagnose</t>
+        </is>
+      </c>
+      <c r="G114" s="15" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="H114" s="15" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I114" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J114" s="16" t="inlineStr">
+        <is>
+          <t>Need one account-level number for whether query mining is too conservative or too loose (all-query CPA ÷ converting-query CPA, bands 1.0–1.5 / 1.5–2.0 / 2.0–2.5 / 2.5+)</t>
+        </is>
+      </c>
+      <c r="K114" s="15" t="inlineStr">
+        <is>
+          <t>Nils Rooijmans script</t>
+        </is>
+      </c>
+      <c r="L114" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M114" s="15" t="n"/>
+      <c r="N114" s="17" t="n"/>
+      <c r="O114" s="15" t="inlineStr">
+        <is>
+          <t>why core: Nils 'Lin Rodnitzky Ratio' script (Nov 2024, updated 2025) in his public catalogue; complements 10/76 which find individual waste but give no account-level verdict.</t>
+        </is>
+      </c>
+      <c r="P114" s="15" t="n"/>
+      <c r="Q114" s="16" t="n"/>
+      <c r="R114" s="15" t="n"/>
+      <c r="S114" s="15" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S91"/>
   <dataValidations count="9">
-    <dataValidation sqref="D2:D91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="D2:D114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Structure,Strategy,Technique,Script,Research,Diagnostic,Setting"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="E2:E91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="E2:E114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Search,Shopping,PMax,All"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="F2:F91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="F2:F114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Setup,Scale,Optimise,Diagnose,Protect"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="G2:G91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="G2:G114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"New,Established,Any"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="H2:H91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H2:H114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"One-off,Weekly,Monthly,As needed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="I2:I114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"P1,P2,P3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="L2:L91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>"Not started,Drafting,Review,Done"</formula1>
+    <dataValidation sqref="L2:L114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+      <formula1>"Not started,Drafting,Review,Done,Proposed,Re-check"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="R2:R91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="R2:R114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Strong,Adequate,Thin"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="S2:S91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="S2:S114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"PASS,FAIL,NEEDS ELIAS"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9112,11 +10745,11 @@
         </is>
       </c>
       <c r="B2" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A2)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A2)</f>
         <v/>
       </c>
       <c r="C2" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A2,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A2,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D2" s="22" t="n"/>
@@ -9126,7 +10759,7 @@
         </is>
       </c>
       <c r="F2" s="22">
-        <f>COUNTIF(Skills!$I$2:$I$91,E2)</f>
+        <f>COUNTIF(Skills!$I$2:$I$114,E2)</f>
         <v/>
       </c>
       <c r="G2" s="22" t="n"/>
@@ -9136,7 +10769,7 @@
         </is>
       </c>
       <c r="I2" s="22">
-        <f>COUNTIF(Skills!$F$2:$F$91,H2)</f>
+        <f>COUNTIF(Skills!$F$2:$F$114,H2)</f>
         <v/>
       </c>
     </row>
@@ -9147,11 +10780,11 @@
         </is>
       </c>
       <c r="B3" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A3)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A3)</f>
         <v/>
       </c>
       <c r="C3" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A3,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A3,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D3" s="22" t="n"/>
@@ -9161,7 +10794,7 @@
         </is>
       </c>
       <c r="F3" s="22">
-        <f>COUNTIF(Skills!$I$2:$I$91,E3)</f>
+        <f>COUNTIF(Skills!$I$2:$I$114,E3)</f>
         <v/>
       </c>
       <c r="G3" s="22" t="n"/>
@@ -9171,7 +10804,7 @@
         </is>
       </c>
       <c r="I3" s="22">
-        <f>COUNTIF(Skills!$F$2:$F$91,H3)</f>
+        <f>COUNTIF(Skills!$F$2:$F$114,H3)</f>
         <v/>
       </c>
     </row>
@@ -9182,11 +10815,11 @@
         </is>
       </c>
       <c r="B4" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A4)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A4,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A4,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D4" s="22" t="n"/>
@@ -9196,7 +10829,7 @@
         </is>
       </c>
       <c r="F4" s="22">
-        <f>COUNTIF(Skills!$I$2:$I$91,E4)</f>
+        <f>COUNTIF(Skills!$I$2:$I$114,E4)</f>
         <v/>
       </c>
       <c r="G4" s="22" t="n"/>
@@ -9206,7 +10839,7 @@
         </is>
       </c>
       <c r="I4" s="22">
-        <f>COUNTIF(Skills!$F$2:$F$91,H4)</f>
+        <f>COUNTIF(Skills!$F$2:$F$114,H4)</f>
         <v/>
       </c>
     </row>
@@ -9217,11 +10850,11 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A5)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A5,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A5,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D5" s="22" t="n"/>
@@ -9234,7 +10867,7 @@
         </is>
       </c>
       <c r="I5" s="22">
-        <f>COUNTIF(Skills!$F$2:$F$91,H5)</f>
+        <f>COUNTIF(Skills!$F$2:$F$114,H5)</f>
         <v/>
       </c>
     </row>
@@ -9245,11 +10878,11 @@
         </is>
       </c>
       <c r="B6" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A6)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A6,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A6,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D6" s="22" t="n"/>
@@ -9262,7 +10895,7 @@
         </is>
       </c>
       <c r="I6" s="22">
-        <f>COUNTIF(Skills!$F$2:$F$91,H6)</f>
+        <f>COUNTIF(Skills!$F$2:$F$114,H6)</f>
         <v/>
       </c>
     </row>
@@ -9273,11 +10906,11 @@
         </is>
       </c>
       <c r="B7" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A7)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A7)</f>
         <v/>
       </c>
       <c r="C7" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A7,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A7,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D7" s="22" t="n"/>
@@ -9294,11 +10927,11 @@
         </is>
       </c>
       <c r="B8" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A8)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A8)</f>
         <v/>
       </c>
       <c r="C8" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A8,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A8,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D8" s="22" t="n"/>
@@ -9315,11 +10948,11 @@
         </is>
       </c>
       <c r="B9" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A9)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A9)</f>
         <v/>
       </c>
       <c r="C9" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A9,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A9,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D9" s="22" t="n"/>
@@ -9336,11 +10969,11 @@
         </is>
       </c>
       <c r="B10" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A10)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A10)</f>
         <v/>
       </c>
       <c r="C10" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A10,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A10,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D10" s="22" t="n"/>
@@ -9357,11 +10990,11 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A11)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A11)</f>
         <v/>
       </c>
       <c r="C11" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A11,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A11,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D11" s="22" t="n"/>
@@ -9378,11 +11011,11 @@
         </is>
       </c>
       <c r="B12" s="22">
-        <f>COUNTIF(Skills!$C$2:$C$91,A12)</f>
+        <f>COUNTIF(Skills!$C$2:$C$114,A12)</f>
         <v/>
       </c>
       <c r="C12" s="22">
-        <f>COUNTIFS(Skills!$C$2:$C$91,A12,Skills!$L$2:$L$91,"Done")</f>
+        <f>COUNTIFS(Skills!$C$2:$C$114,A12,Skills!$L$2:$L$114,"Done")</f>
         <v/>
       </c>
       <c r="D12" s="22" t="n"/>

</xml_diff>

<commit_message>
index: proposed rows 91-113 marked NEEDS ELIAS (go/no-go before building)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSXofh6XbF2HBYEMwgkCSz
</commit_message>
<xml_diff>
--- a/google-ads-skills-index.xlsx
+++ b/google-ads-skills-index.xlsx
@@ -8531,13 +8531,17 @@
       <c r="N92" s="17" t="n"/>
       <c r="O92" s="15" t="inlineStr">
         <is>
-          <t>why core: PPC OS public hub exposes 'Account Audit — 24 diagnostics across 5 modules' and an Account Health Report (Tracking, Campaign Structure, Landing Pages, QS, Ad Quality); TPE #149 lists 13 stacked audits; Hopkins (SEJ 2025) on regular audits; Optmyzr 9-section audit. Library has per-topic diagnostics but no library-level audit row.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: PPC OS public hub exposes 'Account Audit — 24 diagnostics across 5 modules' and an Account Health Report (Tracking, Campaign Structure, Landing Pages, QS, Ad Quality); TPE #149 lists 13 stacked audits; Hopkins (SEJ 2025) on regular audits; Optmyzr 9-section audit. Library has per-topic diagnostics but no library-level audit row.</t>
         </is>
       </c>
       <c r="P92" s="15" t="n"/>
       <c r="Q92" s="16" t="n"/>
       <c r="R92" s="15" t="n"/>
-      <c r="S92" s="15" t="n"/>
+      <c r="S92" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="15" t="n">
@@ -8602,13 +8606,17 @@
       <c r="N93" s="17" t="n"/>
       <c r="O93" s="15" t="inlineStr">
         <is>
-          <t>why core: PPC OS public hub 'Tracking Audit — 50-point check' naming Enhanced Conversions, Consent Mode v2, OCI, attribution model, duplicate actions, primary/secondary; ZATO 'Conversion tracking: why clean data is everything'; Hopkins SEJ 2024 enterprise tracking pitfalls. Rows 47/48 cover two pieces only.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: PPC OS public hub 'Tracking Audit — 50-point check' naming Enhanced Conversions, Consent Mode v2, OCI, attribution model, duplicate actions, primary/secondary; ZATO 'Conversion tracking: why clean data is everything'; Hopkins SEJ 2024 enterprise tracking pitfalls. Rows 47/48 cover two pieces only.</t>
         </is>
       </c>
       <c r="P93" s="15" t="n"/>
       <c r="Q93" s="16" t="n"/>
       <c r="R93" s="15" t="n"/>
-      <c r="S93" s="15" t="n"/>
+      <c r="S93" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="15" t="n">
@@ -8673,13 +8681,17 @@
       <c r="N94" s="17" t="n"/>
       <c r="O94" s="15" t="inlineStr">
         <is>
-          <t>why core: PPC OS 'Performance Analysis' with sample output 'Weekly Review' and 7/30/90/365-day trend windows (TPE #149); Optmyzr audit cadence (weekly health / monthly / quarterly); Adalysis 'how to automate your Google Ads KPI monitoring'.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: PPC OS 'Performance Analysis' with sample output 'Weekly Review' and 7/30/90/365-day trend windows (TPE #149); Optmyzr audit cadence (weekly health / monthly / quarterly); Adalysis 'how to automate your Google Ads KPI monitoring'.</t>
         </is>
       </c>
       <c r="P94" s="15" t="n"/>
       <c r="Q94" s="16" t="n"/>
       <c r="R94" s="15" t="n"/>
-      <c r="S94" s="15" t="n"/>
+      <c r="S94" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="15" t="n">
@@ -8744,13 +8756,17 @@
       <c r="N95" s="17" t="n"/>
       <c r="O95" s="15" t="inlineStr">
         <is>
-          <t>why core: Adalysis 'KPI monitoring diagnosis' series (why does CPC/cost, CTR, clicks, conversions/CVR, impression volume change) plus 'analyze the correct time periods'; PPC OS 'Performance Analysis — the why behind metric shifts'. Rows 84/83/49 cover single causes only.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Adalysis 'KPI monitoring diagnosis' series (why does CPC/cost, CTR, clicks, conversions/CVR, impression volume change) plus 'analyze the correct time periods'; PPC OS 'Performance Analysis — the why behind metric shifts'. Rows 84/83/49 cover single causes only.</t>
         </is>
       </c>
       <c r="P95" s="15" t="n"/>
       <c r="Q95" s="16" t="n"/>
       <c r="R95" s="15" t="n"/>
-      <c r="S95" s="15" t="n"/>
+      <c r="S95" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="15" t="n">
@@ -8815,13 +8831,17 @@
       <c r="N96" s="17" t="n"/>
       <c r="O96" s="15" t="inlineStr">
         <is>
-          <t>why core: Vallaeys 'When to stop using Smart Bidding' (Optmyzr, May 2026; ~50 conv/30d rule, manual CPC + rules alternative); Adalysis 'when to use target vs max CPA/ROAS'; PPC Mastery lists bid strategy choice as a core topic; Hopkins SEJ budget-by-stage. No existing row covers the choice itself.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Vallaeys 'When to stop using Smart Bidding' (Optmyzr, May 2026; ~50 conv/30d rule, manual CPC + rules alternative); Adalysis 'when to use target vs max CPA/ROAS'; PPC Mastery lists bid strategy choice as a core topic; Hopkins SEJ budget-by-stage. No existing row covers the choice itself.</t>
         </is>
       </c>
       <c r="P96" s="15" t="n"/>
       <c r="Q96" s="16" t="n"/>
       <c r="R96" s="15" t="n"/>
-      <c r="S96" s="15" t="n"/>
+      <c r="S96" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="15" t="n">
@@ -8886,13 +8906,17 @@
       <c r="N97" s="17" t="n"/>
       <c r="O97" s="15" t="inlineStr">
         <is>
-          <t>why core: Rhodes 8020agent (profit curve, budget optimisation, break-even ROAS); PPC OS course 'Goal Setting Mastery' + vault 'target calculators'; TPE #144 growth vs efficiency (primary focus + guardrail), TPE #148 LTV flywheel, TPE #149 Phase 1 context questions; Optmyzr ROAS-by-vertical benchmarks (Sep 2026).</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Rhodes 8020agent (profit curve, budget optimisation, break-even ROAS); PPC OS course 'Goal Setting Mastery' + vault 'target calculators'; TPE #144 growth vs efficiency (primary focus + guardrail), TPE #148 LTV flywheel, TPE #149 Phase 1 context questions; Optmyzr ROAS-by-vertical benchmarks (Sep 2026).</t>
         </is>
       </c>
       <c r="P97" s="15" t="n"/>
       <c r="Q97" s="16" t="n"/>
       <c r="R97" s="15" t="n"/>
-      <c r="S97" s="15" t="n"/>
+      <c r="S97" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="15" t="n">
@@ -8957,13 +8981,17 @@
       <c r="N98" s="17" t="n"/>
       <c r="O98" s="15" t="inlineStr">
         <is>
-          <t>why core: Hopkins 'What are learning periods' (SEJ, Dec 2025) and 'Why do budgets overspend with tROAS' (Feb 2026); Adalysis 'what happens when you change your PPC budgets'; PPC Mastery structure-under-Smart-Bidding material. Row 9 only covers campaigns stuck in learning from low volume.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Hopkins 'What are learning periods' (SEJ, Dec 2025) and 'Why do budgets overspend with tROAS' (Feb 2026); Adalysis 'what happens when you change your PPC budgets'; PPC Mastery structure-under-Smart-Bidding material. Row 9 only covers campaigns stuck in learning from low volume.</t>
         </is>
       </c>
       <c r="P98" s="15" t="n"/>
       <c r="Q98" s="16" t="n"/>
       <c r="R98" s="15" t="n"/>
-      <c r="S98" s="15" t="n"/>
+      <c r="S98" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="15" t="n">
@@ -9028,13 +9056,17 @@
       <c r="N99" s="17" t="n"/>
       <c r="O99" s="15" t="inlineStr">
         <is>
-          <t>why core: Geddes 'How to evaluate your AI Max performance' (Adalysis, Aug 2026; broad-match prerequisite, 30 conv/mo, n-gram + asset-source + URL analysis); ZATO has a whole 'AI Max for Search' topic; Cruz 'What are you optimizing for when keywords matter less' (SEL, Apr 2026). No row mentions AI Max.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Geddes 'How to evaluate your AI Max performance' (Adalysis, Aug 2026; broad-match prerequisite, 30 conv/mo, n-gram + asset-source + URL analysis); ZATO has a whole 'AI Max for Search' topic; Cruz 'What are you optimizing for when keywords matter less' (SEL, Apr 2026). No row mentions AI Max.</t>
         </is>
       </c>
       <c r="P99" s="15" t="n"/>
       <c r="Q99" s="16" t="n"/>
       <c r="R99" s="15" t="n"/>
-      <c r="S99" s="15" t="n"/>
+      <c r="S99" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="15" t="n">
@@ -9099,13 +9131,17 @@
       <c r="N100" s="17" t="n"/>
       <c r="O100" s="15" t="inlineStr">
         <is>
-          <t>why core: Rhodes 'products' and 'check-product-data' scripts (GitHub mikerhodesideas/free); Optmyzr 'segment products in Google Shopping ads'; PPC OS 'shopping feed and product optimization'. Row 64 tiers by margin/stock, not by performance.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Rhodes 'products' and 'check-product-data' scripts (GitHub mikerhodesideas/free); Optmyzr 'segment products in Google Shopping ads'; PPC OS 'shopping feed and product optimization'. Row 64 tiers by margin/stock, not by performance.</t>
         </is>
       </c>
       <c r="P100" s="15" t="n"/>
       <c r="Q100" s="16" t="n"/>
       <c r="R100" s="15" t="n"/>
-      <c r="S100" s="15" t="n"/>
+      <c r="S100" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="15" t="n">
@@ -9170,13 +9206,17 @@
       <c r="N101" s="17" t="n"/>
       <c r="O101" s="15" t="inlineStr">
         <is>
-          <t>why core: TPE #145 'Why bid adjustments are dead' (public cheat-sheet by strategy); Adalysis 'how bid adjustments are used by bidding method' and 'how audience bid adjustments work with tCPA/tROAS'. Row 41 covers value rules only.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: TPE #145 'Why bid adjustments are dead' (public cheat-sheet by strategy); Adalysis 'how bid adjustments are used by bidding method' and 'how audience bid adjustments work with tCPA/tROAS'. Row 41 covers value rules only.</t>
         </is>
       </c>
       <c r="P101" s="15" t="n"/>
       <c r="Q101" s="16" t="n"/>
       <c r="R101" s="15" t="n"/>
-      <c r="S101" s="15" t="n"/>
+      <c r="S101" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="15" t="n">
@@ -9241,13 +9281,17 @@
       <c r="N102" s="17" t="n"/>
       <c r="O102" s="15" t="inlineStr">
         <is>
-          <t>why core: PPC OS 'Bids &amp; Budgets — reallocates budgets, validates targets'; Optmyzr 'manage PPC budgets' and 'smart bidding budget caps guide'; Adalysis 'why your campaigns are underspending' and 'IS loss due to budget'; Rhodes 8020agent budget optimiser. Row 71 is only the pacing alert.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: PPC OS 'Bids &amp; Budgets — reallocates budgets, validates targets'; Optmyzr 'manage PPC budgets' and 'smart bidding budget caps guide'; Adalysis 'why your campaigns are underspending' and 'IS loss due to budget'; Rhodes 8020agent budget optimiser. Row 71 is only the pacing alert.</t>
         </is>
       </c>
       <c r="P102" s="15" t="n"/>
       <c r="Q102" s="16" t="n"/>
       <c r="R102" s="15" t="n"/>
-      <c r="S102" s="15" t="n"/>
+      <c r="S102" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="15" t="n">
@@ -9312,13 +9356,17 @@
       <c r="N103" s="17" t="n"/>
       <c r="O103" s="15" t="inlineStr">
         <is>
-          <t>why core: ZATO 'How to scale Google Ads' and 'The physics of PPC'; TPE #147 bottom-up funnel, #144 growth vs efficiency; Hopkins 'From launch to scale: budget strategies for all campaign stages' (SEJ 2024).</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: ZATO 'How to scale Google Ads' and 'The physics of PPC'; TPE #147 bottom-up funnel, #144 growth vs efficiency; Hopkins 'From launch to scale: budget strategies for all campaign stages' (SEJ 2024).</t>
         </is>
       </c>
       <c r="P103" s="15" t="n"/>
       <c r="Q103" s="16" t="n"/>
       <c r="R103" s="15" t="n"/>
-      <c r="S103" s="15" t="n"/>
+      <c r="S103" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="15" t="n">
@@ -9383,13 +9431,17 @@
       <c r="N104" s="17" t="n"/>
       <c r="O104" s="15" t="inlineStr">
         <is>
-          <t>why core: ZATO 'Why isn't my campaign serving — the most asked question in the support forum'; Hopkins 'Why have my ads not got any impressions' (SEJ 2024). Rows 46 and 19 cover under-delivery and low-volume keywords, not non-serving.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: ZATO 'Why isn't my campaign serving — the most asked question in the support forum'; Hopkins 'Why have my ads not got any impressions' (SEJ 2024). Rows 46 and 19 cover under-delivery and low-volume keywords, not non-serving.</t>
         </is>
       </c>
       <c r="P104" s="15" t="n"/>
       <c r="Q104" s="16" t="n"/>
       <c r="R104" s="15" t="n"/>
-      <c r="S104" s="15" t="n"/>
+      <c r="S104" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="15" t="n">
@@ -9454,13 +9506,17 @@
       <c r="N105" s="17" t="n"/>
       <c r="O105" s="15" t="inlineStr">
         <is>
-          <t>why core: Geddes 'Launching a new Search campaign: what to watch in the first month' (Adalysis, 2025); PPC OS 'Search Mastery' public course lists a launch checklist. Rows 87/88 are settings only.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Geddes 'Launching a new Search campaign: what to watch in the first month' (Adalysis, 2025); PPC OS 'Search Mastery' public course lists a launch checklist. Rows 87/88 are settings only.</t>
         </is>
       </c>
       <c r="P105" s="15" t="n"/>
       <c r="Q105" s="16" t="n"/>
       <c r="R105" s="15" t="n"/>
-      <c r="S105" s="15" t="n"/>
+      <c r="S105" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="15" t="n">
@@ -9525,13 +9581,17 @@
       <c r="N106" s="17" t="n"/>
       <c r="O106" s="15" t="inlineStr">
         <is>
-          <t>why core: Adalysis 'understanding and analyzing extension data', 'easily analyze ad extension usage', 'importance of ad extensions', '20 more sitelink ideas'; PPC OS 'Ad Quality (RSAs)' health sub-score. The library has no row on assets/extensions.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Adalysis 'understanding and analyzing extension data', 'easily analyze ad extension usage', 'importance of ad extensions', '20 more sitelink ideas'; PPC OS 'Ad Quality (RSAs)' health sub-score. The library has no row on assets/extensions.</t>
         </is>
       </c>
       <c r="P106" s="15" t="n"/>
       <c r="Q106" s="16" t="n"/>
       <c r="R106" s="15" t="n"/>
-      <c r="S106" s="15" t="n"/>
+      <c r="S106" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="15" t="n">
@@ -9596,13 +9656,17 @@
       <c r="N107" s="17" t="n"/>
       <c r="O107" s="15" t="inlineStr">
         <is>
-          <t>why core: ZATO 'optimize product_type', 'optimize google_product_category', 'why the id attribute matters', 'optimize product descriptions (2026)', 'changing feed providers: roadmap'; PPC OS 'Feeds — titles and secondary attributes'. Rows 65/66 cover rules mechanics and titles only.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: ZATO 'optimize product_type', 'optimize google_product_category', 'why the id attribute matters', 'optimize product descriptions (2026)', 'changing feed providers: roadmap'; PPC OS 'Feeds — titles and secondary attributes'. Rows 65/66 cover rules mechanics and titles only.</t>
         </is>
       </c>
       <c r="P107" s="15" t="n"/>
       <c r="Q107" s="16" t="n"/>
       <c r="R107" s="15" t="n"/>
-      <c r="S107" s="15" t="n"/>
+      <c r="S107" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="15" t="n">
@@ -9667,13 +9731,17 @@
       <c r="N108" s="17" t="n"/>
       <c r="O108" s="15" t="inlineStr">
         <is>
-          <t>why core: ZATO 'How to fix a Merchant Center suspension for misrepresentation', 'tax suspension fix', 'preventing disapprovals and suspensions by mastering compliance'. Row 67 is item-level disapprovals.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: ZATO 'How to fix a Merchant Center suspension for misrepresentation', 'tax suspension fix', 'preventing disapprovals and suspensions by mastering compliance'. Row 67 is item-level disapprovals.</t>
         </is>
       </c>
       <c r="P108" s="15" t="n"/>
       <c r="Q108" s="16" t="n"/>
       <c r="R108" s="15" t="n"/>
-      <c r="S108" s="15" t="n"/>
+      <c r="S108" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="15" t="n">
@@ -9738,13 +9806,17 @@
       <c r="N109" s="17" t="n"/>
       <c r="O109" s="15" t="inlineStr">
         <is>
-          <t>why core: Rhodes 'pmax-assets' script (GitHub); PPC OS 'pMax' skill and 'Performance Max Mastery' course; Hopkins 'Should you use auto-generated creative' (SEJ 2026). Row 58 is structure only.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Rhodes 'pmax-assets' script (GitHub); PPC OS 'pMax' skill and 'Performance Max Mastery' course; Hopkins 'Should you use auto-generated creative' (SEJ 2026). Row 58 is structure only.</t>
         </is>
       </c>
       <c r="P109" s="15" t="n"/>
       <c r="Q109" s="16" t="n"/>
       <c r="R109" s="15" t="n"/>
-      <c r="S109" s="15" t="n"/>
+      <c r="S109" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="15" t="n">
@@ -9809,13 +9881,17 @@
       <c r="N110" s="17" t="n"/>
       <c r="O110" s="15" t="inlineStr">
         <is>
-          <t>why core: Hopkins 'How to identify and solve click fraud' (SEJ, Apr 2026); Optmyzr 'Protect Smart Bidding from spam conversions' (Jul 2026, method only, vendor byline); ZATO clean-data post. Row 44 covers data exclusions after the fact, not detection.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Hopkins 'How to identify and solve click fraud' (SEJ, Apr 2026); Optmyzr 'Protect Smart Bidding from spam conversions' (Jul 2026, method only, vendor byline); ZATO clean-data post. Row 44 covers data exclusions after the fact, not detection.</t>
         </is>
       </c>
       <c r="P110" s="15" t="n"/>
       <c r="Q110" s="16" t="n"/>
       <c r="R110" s="15" t="n"/>
-      <c r="S110" s="15" t="n"/>
+      <c r="S110" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="15" t="n">
@@ -9880,13 +9956,17 @@
       <c r="N111" s="17" t="n"/>
       <c r="O111" s="15" t="inlineStr">
         <is>
-          <t>why core: PPC OS 'Landing Pages — 6-pillar structural audit' and 'Landing Page Mastery' course; Adalysis 'test landing pages and ads together', 'customer journey testing'; Rhodes 'landing-page' script; Optmyzr 'PPC landing page AI signal problem'. Row 36 is the QS LPE component only.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: PPC OS 'Landing Pages — 6-pillar structural audit' and 'Landing Page Mastery' course; Adalysis 'test landing pages and ads together', 'customer journey testing'; Rhodes 'landing-page' script; Optmyzr 'PPC landing page AI signal problem'. Row 36 is the QS LPE component only.</t>
         </is>
       </c>
       <c r="P111" s="15" t="n"/>
       <c r="Q111" s="16" t="n"/>
       <c r="R111" s="15" t="n"/>
-      <c r="S111" s="15" t="n"/>
+      <c r="S111" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="15" t="n">
@@ -9951,13 +10031,17 @@
       <c r="N112" s="17" t="n"/>
       <c r="O112" s="15" t="inlineStr">
         <is>
-          <t>why core: Vallaeys 'Automation layering is driving PPC' (SEL) and canon lists it among his strongest topics; Hopkins 'How do I keep control as platforms automate my account' (SEJ, Sep 2026); Optmyzr 72,358-account manual-work study (Sep 2026). Row 77 is rules-vs-scripts tool choice, not the layering strategy.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Vallaeys 'Automation layering is driving PPC' (SEL) and canon lists it among his strongest topics; Hopkins 'How do I keep control as platforms automate my account' (SEJ, Sep 2026); Optmyzr 72,358-account manual-work study (Sep 2026). Row 77 is rules-vs-scripts tool choice, not the layering strategy.</t>
         </is>
       </c>
       <c r="P112" s="15" t="n"/>
       <c r="Q112" s="16" t="n"/>
       <c r="R112" s="15" t="n"/>
-      <c r="S112" s="15" t="n"/>
+      <c r="S112" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="15" t="n">
@@ -10022,13 +10106,17 @@
       <c r="N113" s="17" t="n"/>
       <c r="O113" s="15" t="inlineStr">
         <is>
-          <t>why core: Nils 'Change history alerts' script (public catalogue); Hopkins Sep 2026 on keeping control under automation. Row 78 only opts out of auto-apply; it does not monitor what changed.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Nils 'Change history alerts' script (public catalogue); Hopkins Sep 2026 on keeping control under automation. Row 78 only opts out of auto-apply; it does not monitor what changed.</t>
         </is>
       </c>
       <c r="P113" s="15" t="n"/>
       <c r="Q113" s="16" t="n"/>
       <c r="R113" s="15" t="n"/>
-      <c r="S113" s="15" t="n"/>
+      <c r="S113" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="15" t="n">
@@ -10093,13 +10181,17 @@
       <c r="N114" s="17" t="n"/>
       <c r="O114" s="15" t="inlineStr">
         <is>
-          <t>why core: Nils 'Lin Rodnitzky Ratio' script (Nov 2024, updated 2025) in his public catalogue; complements 10/76 which find individual waste but give no account-level verdict.</t>
+          <t>Proposed in the Phase 2 coverage pass — needs Elias go/no-go before building. why core: Nils 'Lin Rodnitzky Ratio' script (Nov 2024, updated 2025) in his public catalogue; complements 10/76 which find individual waste but give no account-level verdict.</t>
         </is>
       </c>
       <c r="P114" s="15" t="n"/>
       <c r="Q114" s="16" t="n"/>
       <c r="R114" s="15" t="n"/>
-      <c r="S114" s="15" t="n"/>
+      <c r="S114" s="15" t="inlineStr">
+        <is>
+          <t>NEEDS ELIAS</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S91"/>

</xml_diff>